<commit_message>
new excel format added, improved UI parts and bug fixes
</commit_message>
<xml_diff>
--- a/static/roster_format.xlsx
+++ b/static/roster_format.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Route Assignments" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,32 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000F1A2E"/>
-        <bgColor rgb="000F1A2E"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -58,32 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D0D0D0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D0D0D0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D0D0D0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D0D0D0"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -449,286 +413,60 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Driver Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Vehicle Code</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Vehicle Plate</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Route</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Staging</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Pad</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Wave Time</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-      <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
-      <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
-      <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-      <c r="B11" s="2" t="inlineStr"/>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr"/>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-      <c r="B13" s="2" t="inlineStr"/>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
-      <c r="B14" s="2" t="inlineStr"/>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-      <c r="B15" s="2" t="inlineStr"/>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr"/>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
-      <c r="B17" s="2" t="inlineStr"/>
-      <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
-      <c r="B18" s="2" t="inlineStr"/>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-      <c r="B19" s="2" t="inlineStr"/>
-      <c r="C19" s="2" t="inlineStr"/>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-      <c r="B20" s="2" t="inlineStr"/>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
-      <c r="B21" s="2" t="inlineStr"/>
-      <c r="C21" s="2" t="inlineStr"/>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Route code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>DSP</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Transporter Id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Driver name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Route progress</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Delivery service type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Route duration</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>All stops</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Stops completed</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Not started stops</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>